<commit_message>
feat: evaluation updates and test case improvements
</commit_message>
<xml_diff>
--- a/src/docs/testfile.xlsx
+++ b/src/docs/testfile.xlsx
@@ -1,16 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/santhosh/Desktop/podhealth/eval-engine/src/docs/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3D03CA-87EF-E24C-A20B-15814A97DEF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{26601BB4-00BE-4C87-B11C-DD96B91BEEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -39,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="109">
   <si>
     <t xml:space="preserve"> POD HEALTH — AI Data Agent Evaluation Tracker</t>
   </si>
@@ -98,13 +93,150 @@
     <t>Can you tell me how my child's overall health is progressing?</t>
   </si>
   <si>
-    <t>- Summarises recent health trends across all domains (physical, mental, behavioural)
-- References latest health log entries
-- Highlights improvements or regressions
-- Provides actionable next steps</t>
+    <t xml:space="preserve">- Provides an overall summary of the child’s current health status
+-Mentions ongoing care, monitoring, or key conditions if available
+-Uses available data without making unsupported claims
+- Gives a clear and helpful parent-friendly explanation
+</t>
   </si>
   <si>
     <t>Qualitative</t>
+  </si>
+  <si>
+    <t>Q-002</t>
+  </si>
+  <si>
+    <t>Can you give me a list of all the active medications my child is taking and the side effects of those medications?</t>
+  </si>
+  <si>
+    <t>- Lists every active medication by name if available
+- Includes dosage or basic details if present
+-Mentions  side effects for medications
+-Provides clear and structured explination
+-Does not assume missing details like frequency or interactions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantitative
+</t>
+  </si>
+  <si>
+    <t>Q-003</t>
+  </si>
+  <si>
+    <t>Can you give me some latest research on Autism, ADHD, Depression and Anxiety?</t>
+  </si>
+  <si>
+    <t>- Provides a general overview or recent insights for Autism, ADHD, Depression, and Anxiety
+- Covers each condition clearly and keeps them distinct
+- Gives relevant and parent-friendly explanation
+- Includes research-based or medically relevant information if available
+- Avoids unsupported, overly specific, or fabricated claims</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Qualitative
+</t>
+  </si>
+  <si>
+    <t>Q-004</t>
+  </si>
+  <si>
+    <t>Can you summarize the last document I uploaded?</t>
+  </si>
+  <si>
+    <t>- Identifies the most recent or relevant document if available
+- Provides a clear summary of key points from the document
+- Avoids adding information not present in the document
+- Gives a structured and easy-to-understand explanation</t>
+  </si>
+  <si>
+    <t>Q-005</t>
+  </si>
+  <si>
+    <t>Can you summarize my child's life logs?</t>
+  </si>
+  <si>
+    <t>- Summarizes life log entries if they are available
+- If no life logs are present, clearly states that no logs are available
+- Avoids inventing activities, events, or patterns that are not in the data
+- Gives a clear and parent-friendly response
+- Mentions trends or patterns only when supported by actual logged data</t>
+  </si>
+  <si>
+    <t>Q-006</t>
+  </si>
+  <si>
+    <t>Can you list the key health observations recorded for my child in the past week?</t>
+  </si>
+  <si>
+    <t>- Summarizes key health observations from the past week if available
+- If no observations are present, indicates that no recent data or logs are available
+- Accepts responses that explain absence of data in different ways
+- Highlights important updates, symptoms, or events when data exists
+- Avoids adding information not present in the records
+- Keeps the response clear and parent-friendly</t>
+  </si>
+  <si>
+    <t>Q-007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can you identify any potential concerns based on my child's recent health records?
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Reviews available health records or logs if present
+- Identifies potential concerns only if supported by data
+- If no concerns or no data, clearly states that nothing concerning is found or data is unavailable
+- Explains why a concern may be important when identified
+- Avoids making unsupported or speculative claims
+- Keeps explanation clear and parent-friendly
+- May suggest consulting a professional if needed
+</t>
+  </si>
+  <si>
+    <t>Q-008</t>
+  </si>
+  <si>
+    <t>Can you summarize how my child has been doing over the past few days based on the logs?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Summarizes how the child has been doing over the past few days if recent log data is available
+- Highlights notable observations, activities, behaviors, or changes mentioned in the logs
+- If no recent logs are available, acknowledges that there is no or limited data to summarize (phrases like "no logs", "no data", or similar are acceptable)
+- Avoids generating information not present in the logs
+- Keeps the response clear and parent-friendly
+</t>
+  </si>
+  <si>
+    <t>Q-009</t>
+  </si>
+  <si>
+    <t>Has my child shown any positive progress
+ in their daily activities recently?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Reviews recent activity logs if available
+- Identifies signs of improvement or positive progress when supported by data
+- If no recent logs or data are available, clearly states that no recent progress can be determined
+- References relevant entries or timing when data exists
+- Avoids making unsupported or speculative conclusions
+- Keeps the explanation clear and parent-friendly
+</t>
+  </si>
+  <si>
+    <t>Q-010</t>
+  </si>
+  <si>
+    <t>Were there any moments where my child
+ seemed calmer or happier during the day?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Reviews mood or activity logs if available
+- Identifies moments of calmer, happier, or more positive emotional state only when supported by data
+- If no relevant logs or observations are available, clearly states that this cannot be determined from recent records
+- References relevant observations or timing when data exists
+- Avoids speculation or unsupported conclusions
+- Keeps the response clear and parent-friendly
+</t>
   </si>
   <si>
     <t>📊  Evaluation Score Summary</t>
@@ -291,7 +423,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -304,53 +436,45 @@
       <sz val="16"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF555555"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="15"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -433,7 +557,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -489,10 +613,15 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -505,7 +634,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -515,6 +643,8 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -842,8 +972,8 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:O14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -858,46 +988,46 @@
     <col min="14" max="15" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="21" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-    </row>
-    <row r="2" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="19" t="s">
+    <row r="1" spans="1:15" ht="39.950000000000003" customHeight="1">
+      <c r="A1" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+    </row>
+    <row r="2" spans="1:15" ht="20.100000000000001" customHeight="1">
+      <c r="A2" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
-      <c r="G2" s="20"/>
-      <c r="H2" s="20"/>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20"/>
-      <c r="L2" s="20"/>
-      <c r="M2" s="20"/>
-      <c r="N2" s="20"/>
-      <c r="O2" s="20"/>
-    </row>
-    <row r="3" spans="1:15" ht="14" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="29"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+      <c r="L2" s="29"/>
+      <c r="M2" s="29"/>
+      <c r="N2" s="29"/>
+      <c r="O2" s="29"/>
+    </row>
+    <row r="3" spans="1:15" ht="14.1" customHeight="1"/>
+    <row r="4" spans="1:15" ht="36" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -944,7 +1074,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" ht="80.099999999999994" customHeight="1">
       <c r="A5" s="5">
         <v>1</v>
       </c>
@@ -977,16 +1107,229 @@
       <c r="N5" s="5"/>
       <c r="O5" s="5"/>
     </row>
-    <row r="6" spans="1:15" ht="80" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="7" spans="1:15" ht="80" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="8" spans="1:15" ht="80" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="9" spans="1:15" ht="80" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="6" spans="1:15" ht="80.099999999999994" customHeight="1">
+      <c r="A6" s="8">
+        <v>2</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="9" t="str">
+        <f>IF(I6="","",I6/10)</f>
+        <v/>
+      </c>
+      <c r="K6" s="8" t="str">
+        <f>IF(I6="","",IF(I6&gt;=7,"Pass",IF(I6&gt;=4,"Partial","Fail")))</f>
+        <v/>
+      </c>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="1:15" ht="80.099999999999994" customHeight="1">
+      <c r="A7" s="5">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="7" t="str">
+        <f>IF(I7="","",I7/10)</f>
+        <v/>
+      </c>
+      <c r="K7" s="5" t="str">
+        <f>IF(I7="","",IF(I7&gt;=7,"Pass",IF(I7&gt;=4,"Partial","Fail")))</f>
+        <v/>
+      </c>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+    </row>
+    <row r="8" spans="1:15" ht="80.099999999999994" customHeight="1">
+      <c r="A8" s="8">
+        <v>4</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="9" t="str">
+        <f>IF(I8="","",I8/10)</f>
+        <v/>
+      </c>
+      <c r="K8" s="8" t="str">
+        <f>IF(I8="","",IF(I8&gt;=7,"Pass",IF(I8&gt;=4,"Partial","Fail")))</f>
+        <v/>
+      </c>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" spans="1:15" ht="80.099999999999994" customHeight="1">
+      <c r="A9" s="5">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="7" t="str">
+        <f>IF(I9="","",I9/10)</f>
+        <v/>
+      </c>
+      <c r="K9" s="5" t="str">
+        <f>IF(I9="","",IF(I9&gt;=7,"Pass",IF(I9&gt;=4,"Partial","Fail")))</f>
+        <v/>
+      </c>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+    </row>
+    <row r="10" spans="1:15" ht="152.25">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="183">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="152.25">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="137.25">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="183">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <conditionalFormatting sqref="I5">
+  <conditionalFormatting sqref="I5:I81">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -998,7 +1341,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5">
+  <conditionalFormatting sqref="K5:K81">
     <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
       <formula>"Pass"</formula>
     </cfRule>
@@ -1010,17 +1353,17 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="whole" showErrorMessage="1" errorTitle="Invalid Score" error="Enter a number between 0 and 10" sqref="I5" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="whole" showErrorMessage="1" errorTitle="Invalid Score" error="Enter a number between 0 and 10" sqref="I5:I81" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
       <formula2>10</formula2>
     </dataValidation>
-    <dataValidation type="list" sqref="K5" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="K5:K81" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Pass,Fail,Partial"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="N5" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" sqref="N5:N81" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="O5" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" sqref="O5:O81" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1032,7 +1375,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -1040,51 +1383,51 @@
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-    </row>
-    <row r="3" spans="1:8" ht="32" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="38.1" customHeight="1">
+      <c r="A1" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+    </row>
+    <row r="3" spans="1:8" ht="32.1" customHeight="1">
       <c r="A3" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>11</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="G3" s="10" t="s">
         <v>16</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="24" customHeight="1">
       <c r="A4" s="5" t="str">
         <f>'Test Cases'!B5</f>
         <v>Q-001</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="C4" s="5">
         <f>'Test Cases'!I5</f>
@@ -1111,182 +1454,182 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
+    <row r="5" spans="1:8" ht="24" customHeight="1">
+      <c r="A5" s="8" t="str">
+        <f>'Test Cases'!B6</f>
+        <v>Q-002</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D5" s="9" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E5" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F5" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G5" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H5" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
+        <v>57</v>
+      </c>
+      <c r="C5" s="8">
+        <f>'Test Cases'!I6</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="9" t="str">
+        <f>'Test Cases'!J6</f>
+        <v/>
+      </c>
+      <c r="E5" s="8" t="str">
+        <f>'Test Cases'!K6</f>
+        <v/>
+      </c>
+      <c r="F5" s="8">
+        <f>'Test Cases'!N6</f>
+        <v>0</v>
+      </c>
+      <c r="G5" s="8">
+        <f>'Test Cases'!O6</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="8">
+        <f>'Test Cases'!M6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="24" customHeight="1">
+      <c r="A6" s="5" t="str">
+        <f>'Test Cases'!B7</f>
+        <v>Q-003</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D6" s="7" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E6" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F6" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G6" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H6" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
+        <v>58</v>
+      </c>
+      <c r="C6" s="5">
+        <f>'Test Cases'!I7</f>
+        <v>0</v>
+      </c>
+      <c r="D6" s="7" t="str">
+        <f>'Test Cases'!J7</f>
+        <v/>
+      </c>
+      <c r="E6" s="5" t="str">
+        <f>'Test Cases'!K7</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>'Test Cases'!N7</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="5">
+        <f>'Test Cases'!O7</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="5">
+        <f>'Test Cases'!M7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="24" customHeight="1">
+      <c r="A7" s="8" t="str">
+        <f>'Test Cases'!B8</f>
+        <v>Q-004</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D7" s="9" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E7" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F7" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G7" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H7" s="8" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
+        <v>59</v>
+      </c>
+      <c r="C7" s="8">
+        <f>'Test Cases'!I8</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="9" t="str">
+        <f>'Test Cases'!J8</f>
+        <v/>
+      </c>
+      <c r="E7" s="8" t="str">
+        <f>'Test Cases'!K8</f>
+        <v/>
+      </c>
+      <c r="F7" s="8">
+        <f>'Test Cases'!N8</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="8">
+        <f>'Test Cases'!O8</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="8">
+        <f>'Test Cases'!M8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="24" customHeight="1">
+      <c r="A8" s="5" t="str">
+        <f>'Test Cases'!B9</f>
+        <v>Q-005</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="D8" s="7" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="E8" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="F8" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="G8" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-      <c r="H8" s="5" t="e">
-        <f>'Test Cases'!#REF!</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="22" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="20"/>
-      <c r="C9" s="11" t="e">
+        <v>60</v>
+      </c>
+      <c r="C8" s="5">
+        <f>'Test Cases'!I9</f>
+        <v>0</v>
+      </c>
+      <c r="D8" s="7" t="str">
+        <f>'Test Cases'!J9</f>
+        <v/>
+      </c>
+      <c r="E8" s="5" t="str">
+        <f>'Test Cases'!K9</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>'Test Cases'!N9</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="5">
+        <f>'Test Cases'!O9</f>
+        <v>0</v>
+      </c>
+      <c r="H8" s="5">
+        <f>'Test Cases'!M9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="27.95" customHeight="1">
+      <c r="A9" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="29"/>
+      <c r="C9" s="11">
         <f>AVERAGE(C4:C8)</f>
-        <v>#REF!</v>
+        <v>0</v>
       </c>
       <c r="D9" s="12" t="e">
         <f>AVERAGE(D4:D8)</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="13" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="B11" s="14">
         <f>COUNTIF(E4:E8,"Pass")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8">
       <c r="A12" s="13" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="B12" s="14">
         <f>COUNTIF(E4:E8,"Partial")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8">
       <c r="A13" s="13" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="B13" s="14">
         <f>COUNTIF(E4:E8,"Fail")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8">
       <c r="A14" s="13" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="B14" s="14">
         <f>COUNTIF(F4:F8,"Yes")</f>
@@ -1305,7 +1648,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -1314,37 +1657,37 @@
     <col min="6" max="6" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-    </row>
-    <row r="3" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="38.1" customHeight="1">
+      <c r="A1" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+    </row>
+    <row r="3" spans="1:6" ht="27.95" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>38</v>
+        <v>67</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="21.95" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -1352,7 +1695,7 @@
       <c r="E4" s="5"/>
       <c r="F4" s="5"/>
     </row>
-    <row r="5" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="21.95" customHeight="1">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1360,7 +1703,7 @@
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
     </row>
-    <row r="6" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="21.95" customHeight="1">
       <c r="A6" s="5"/>
       <c r="B6" s="5"/>
       <c r="C6" s="5"/>
@@ -1368,7 +1711,7 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="21.95" customHeight="1">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -1376,7 +1719,7 @@
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
     </row>
-    <row r="8" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="21.95" customHeight="1">
       <c r="A8" s="5"/>
       <c r="B8" s="5"/>
       <c r="C8" s="5"/>
@@ -1384,7 +1727,7 @@
       <c r="E8" s="5"/>
       <c r="F8" s="5"/>
     </row>
-    <row r="9" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="21.95" customHeight="1">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -1392,7 +1735,7 @@
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
     </row>
-    <row r="10" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="21.95" customHeight="1">
       <c r="A10" s="5"/>
       <c r="B10" s="5"/>
       <c r="C10" s="5"/>
@@ -1400,7 +1743,7 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
     </row>
-    <row r="11" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="21.95" customHeight="1">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -1408,7 +1751,7 @@
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
     </row>
-    <row r="12" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="21.95" customHeight="1">
       <c r="A12" s="5"/>
       <c r="B12" s="5"/>
       <c r="C12" s="5"/>
@@ -1416,7 +1759,7 @@
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
     </row>
-    <row r="13" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="21.95" customHeight="1">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -1424,7 +1767,7 @@
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
     </row>
-    <row r="14" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" ht="21.95" customHeight="1">
       <c r="A14" s="5"/>
       <c r="B14" s="5"/>
       <c r="C14" s="5"/>
@@ -1432,7 +1775,7 @@
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
     </row>
-    <row r="15" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="21.95" customHeight="1">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -1440,7 +1783,7 @@
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
     </row>
-    <row r="16" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="21.95" customHeight="1">
       <c r="A16" s="5"/>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -1448,7 +1791,7 @@
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
     </row>
-    <row r="17" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="21.95" customHeight="1">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -1456,7 +1799,7 @@
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
     </row>
-    <row r="18" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="21.95" customHeight="1">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -1464,7 +1807,7 @@
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
     </row>
-    <row r="19" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="21.95" customHeight="1">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -1483,7 +1826,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -1491,161 +1834,161 @@
     <col min="4" max="4" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-    </row>
-    <row r="3" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-    </row>
-    <row r="4" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="38.1" customHeight="1">
+      <c r="A1" s="24" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+    </row>
+    <row r="3" spans="1:4" ht="24" customHeight="1">
+      <c r="A3" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+    </row>
+    <row r="4" spans="1:4" ht="38.1" customHeight="1">
       <c r="A4" s="15" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="D4" s="25"/>
-    </row>
-    <row r="5" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+      <c r="D4" s="30"/>
+    </row>
+    <row r="5" spans="1:4" ht="38.1" customHeight="1">
       <c r="A5" s="15" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" s="25"/>
-    </row>
-    <row r="6" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
+        <v>80</v>
+      </c>
+      <c r="D5" s="30"/>
+    </row>
+    <row r="6" spans="1:4" ht="38.1" customHeight="1">
       <c r="A6" s="15" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="D6" s="25"/>
-    </row>
-    <row r="7" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
+        <v>83</v>
+      </c>
+      <c r="D6" s="30"/>
+    </row>
+    <row r="7" spans="1:4" ht="38.1" customHeight="1">
       <c r="A7" s="15" t="s">
-        <v>55</v>
+        <v>84</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>56</v>
+        <v>85</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="D7" s="25"/>
-    </row>
-    <row r="8" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
+        <v>86</v>
+      </c>
+      <c r="D7" s="30"/>
+    </row>
+    <row r="8" spans="1:4" ht="38.1" customHeight="1">
       <c r="A8" s="15" t="s">
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>59</v>
+        <v>88</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="25"/>
-    </row>
-    <row r="9" spans="1:4" ht="38" customHeight="1" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+      <c r="D8" s="30"/>
+    </row>
+    <row r="9" spans="1:4" ht="38.1" customHeight="1">
       <c r="A9" s="15" t="s">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>63</v>
-      </c>
-      <c r="D9" s="25"/>
-    </row>
-    <row r="11" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+        <v>92</v>
+      </c>
+      <c r="D9" s="30"/>
+    </row>
+    <row r="11" spans="1:4" ht="24" customHeight="1">
       <c r="A11" s="28" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-    </row>
-    <row r="12" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+    </row>
+    <row r="12" spans="1:4" ht="27.95" customHeight="1">
       <c r="A12" s="17" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="D12" s="25"/>
-    </row>
-    <row r="13" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+        <v>95</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="D12" s="30"/>
+    </row>
+    <row r="13" spans="1:4" ht="27.95" customHeight="1">
       <c r="A13" s="17" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="D13" s="25"/>
-    </row>
-    <row r="14" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="D13" s="30"/>
+    </row>
+    <row r="14" spans="1:4" ht="27.95" customHeight="1">
       <c r="A14" s="17" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="C14" s="24" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" s="25"/>
-    </row>
-    <row r="15" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="D14" s="30"/>
+    </row>
+    <row r="15" spans="1:4" ht="27.95" customHeight="1">
       <c r="A15" s="17" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>75</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="D15" s="25"/>
-    </row>
-    <row r="16" spans="1:4" ht="28" customHeight="1" x14ac:dyDescent="0.2">
+        <v>104</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="D15" s="30"/>
+    </row>
+    <row r="16" spans="1:4" ht="27.95" customHeight="1">
       <c r="A16" s="17" t="s">
-        <v>77</v>
+        <v>106</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="C16" s="24" t="s">
-        <v>79</v>
-      </c>
-      <c r="D16" s="25"/>
+        <v>107</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="D16" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>